<commit_message>
refactor(ui): streamline accountant & director navigation, simplify trip list
- Rename "Đối tác" → "Nhà thầu", "Đối soát" → "Ghép chuyến" across roles
- Remove unused sidebar items (Nhập từ Excel, Nhập bảng giá, Cung đường)
- Simplify TripList to 2 status groups (chờ đối soát / đã khớp)
- Reorder dashboard KPIs to surface pending work first
- Remove director quick-actions section
- Update docs and add AGENTS.md

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/2.GLORY SHANGHAI- 2612N.xlsx
+++ b/docs/2.GLORY SHANGHAI- 2612N.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\2026\THÁNG 4\CHECK SJJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A5102C-1055-49C9-9193-79D8CB5ADAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0F5405-5CFC-4A43-B264-098AC82FD41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4621" uniqueCount="706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4498" uniqueCount="706">
   <si>
     <t>Vị trí hộp</t>
   </si>
@@ -2219,12 +2219,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -2276,7 +2282,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2323,11 +2329,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2335,14 +2348,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2630,8 +2635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4647F203-D603-477A-835D-7581165CB706}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:AA275"/>
+  <dimension ref="A1:AA149"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="1"/>
@@ -2758,13 +2762,13 @@
       <c r="C4" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="20" t="s">
         <v>227</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="20" t="s">
         <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -2810,20 +2814,20 @@
         <v>26400000</v>
       </c>
     </row>
-    <row r="5" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="21" t="s">
         <v>464</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>414</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -2878,20 +2882,20 @@
         <v>9680000</v>
       </c>
     </row>
-    <row r="6" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="21" t="s">
         <v>465</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>415</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G6" s="3" t="s">
@@ -2946,20 +2950,20 @@
         <v>15372000</v>
       </c>
     </row>
-    <row r="7" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>3</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="21" t="s">
         <v>466</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>416</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -3015,20 +3019,20 @@
         <v>51452000</v>
       </c>
     </row>
-    <row r="8" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>4</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="21" t="s">
         <v>467</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>417</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -3080,20 +3084,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="9" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="21" t="s">
         <v>468</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>418</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -3145,20 +3149,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="10" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="21" t="s">
         <v>469</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>419</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -3210,20 +3214,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="11" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>7</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="21" t="s">
         <v>470</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>420</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -3275,20 +3279,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="12" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>8</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="21" t="s">
         <v>471</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>421</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G12" s="3" t="s">
@@ -3340,20 +3344,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="13" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="21" t="s">
         <v>472</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>422</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -3405,20 +3409,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="14" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>10</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="21" t="s">
         <v>473</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -3477,13 +3481,13 @@
       <c r="C15" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="21" t="s">
         <v>474</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -3535,20 +3539,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="16" spans="1:27" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>12</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="D16" s="21" t="s">
         <v>475</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>425</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -3600,20 +3604,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="17" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B17" s="3">
         <v>13</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="21" t="s">
         <v>476</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>426</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -3665,20 +3669,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="18" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B18" s="3">
         <v>14</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="D18" s="21" t="s">
         <v>477</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>427</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -3737,13 +3741,13 @@
       <c r="C19" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="21" t="s">
         <v>478</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>428</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -3795,20 +3799,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="20" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B20" s="3">
         <v>16</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="21" t="s">
         <v>479</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -3860,20 +3864,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="21" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B21" s="3">
         <v>17</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="21" t="s">
         <v>480</v>
       </c>
       <c r="E21" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -3932,13 +3936,13 @@
       <c r="C22" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="21" t="s">
         <v>481</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>431</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -3990,20 +3994,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="23" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B23" s="3">
         <v>19</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="11" t="s">
+      <c r="D23" s="21" t="s">
         <v>482</v>
       </c>
       <c r="E23" s="11" t="s">
         <v>432</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G23" s="3" t="s">
@@ -4055,20 +4059,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="24" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B24" s="3">
         <v>20</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="21" t="s">
         <v>483</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>433</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -4127,13 +4131,13 @@
       <c r="C25" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="21" t="s">
         <v>484</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>434</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -4185,20 +4189,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="26" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B26" s="3">
         <v>22</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="D26" s="21" t="s">
         <v>485</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>435</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G26" s="3" t="s">
@@ -4250,20 +4254,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="27" spans="2:24" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B27" s="3">
         <v>23</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D27" s="11" t="s">
+      <c r="D27" s="21" t="s">
         <v>486</v>
       </c>
       <c r="E27" s="11" t="s">
         <v>436</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -4299,20 +4303,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="28" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B28" s="3">
         <v>24</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="21" t="s">
         <v>487</v>
       </c>
       <c r="E28" s="11" t="s">
         <v>437</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G28" s="3" t="s">
@@ -4344,20 +4348,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="29" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B29" s="3">
         <v>25</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="21" t="s">
         <v>488</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>438</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G29" s="3" t="s">
@@ -4389,20 +4393,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="30" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B30" s="3">
         <v>26</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="21" t="s">
         <v>489</v>
       </c>
       <c r="E30" s="11" t="s">
         <v>439</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -4434,20 +4438,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="31" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B31" s="3">
         <v>27</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="21" t="s">
         <v>490</v>
       </c>
       <c r="E31" s="11" t="s">
         <v>440</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -4479,20 +4483,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="32" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B32" s="3">
         <v>28</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D32" s="11" t="s">
+      <c r="D32" s="21" t="s">
         <v>491</v>
       </c>
       <c r="E32" s="11" t="s">
         <v>441</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -4524,20 +4528,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="33" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B33" s="3">
         <v>29</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="21" t="s">
         <v>492</v>
       </c>
       <c r="E33" s="11" t="s">
         <v>442</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -4576,13 +4580,13 @@
       <c r="C34" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D34" s="11" t="s">
+      <c r="D34" s="21" t="s">
         <v>493</v>
       </c>
       <c r="E34" s="11" t="s">
         <v>443</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -4614,20 +4618,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="35" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B35" s="3">
         <v>31</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="D35" s="21" t="s">
         <v>494</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>444</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -4658,20 +4662,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="36" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B36" s="3">
         <v>32</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D36" s="11" t="s">
+      <c r="D36" s="21" t="s">
         <v>495</v>
       </c>
       <c r="E36" s="11" t="s">
         <v>445</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G36" s="3" t="s">
@@ -4702,20 +4706,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="37" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B37" s="3">
         <v>33</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="21" t="s">
         <v>496</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>446</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G37" s="3" t="s">
@@ -4746,20 +4750,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="38" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B38" s="3">
         <v>34</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="D38" s="21" t="s">
         <v>497</v>
       </c>
       <c r="E38" s="11" t="s">
         <v>447</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G38" s="3" t="s">
@@ -4797,13 +4801,13 @@
       <c r="C39" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D39" s="11" t="s">
+      <c r="D39" s="21" t="s">
         <v>498</v>
       </c>
       <c r="E39" s="11" t="s">
         <v>448</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G39" s="3" t="s">
@@ -4834,20 +4838,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="40" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B40" s="3">
         <v>36</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="21" t="s">
         <v>499</v>
       </c>
       <c r="E40" s="11" t="s">
         <v>449</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -4878,20 +4882,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="41" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B41" s="3">
         <v>37</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="21" t="s">
         <v>500</v>
       </c>
       <c r="E41" s="11" t="s">
         <v>450</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G41" s="3" t="s">
@@ -4922,20 +4926,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="42" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B42" s="3">
         <v>38</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="21" t="s">
         <v>501</v>
       </c>
       <c r="E42" s="11" t="s">
         <v>451</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G42" s="3" t="s">
@@ -4973,13 +4977,13 @@
       <c r="C43" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="21" t="s">
         <v>502</v>
       </c>
       <c r="E43" s="11" t="s">
         <v>452</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G43" s="3" t="s">
@@ -5017,13 +5021,13 @@
       <c r="C44" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="21" t="s">
         <v>503</v>
       </c>
       <c r="E44" s="11" t="s">
         <v>453</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="F44" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G44" s="3" t="s">
@@ -5054,20 +5058,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="45" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B45" s="3">
         <v>41</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D45" s="11" t="s">
+      <c r="D45" s="21" t="s">
         <v>504</v>
       </c>
       <c r="E45" s="11" t="s">
         <v>454</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="F45" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G45" s="3" t="s">
@@ -5105,13 +5109,13 @@
       <c r="C46" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="21" t="s">
         <v>505</v>
       </c>
       <c r="E46" s="11" t="s">
         <v>455</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="F46" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G46" s="3" t="s">
@@ -5142,20 +5146,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="47" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B47" s="3">
         <v>43</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="D47" s="21" t="s">
         <v>506</v>
       </c>
       <c r="E47" s="11" t="s">
         <v>456</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="F47" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G47" s="3" t="s">
@@ -5186,20 +5190,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="48" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B48" s="3">
         <v>44</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D48" s="11" t="s">
+      <c r="D48" s="21" t="s">
         <v>507</v>
       </c>
       <c r="E48" s="11" t="s">
         <v>457</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="F48" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G48" s="3" t="s">
@@ -5230,20 +5234,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="49" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B49" s="3">
         <v>45</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D49" s="21" t="s">
         <v>508</v>
       </c>
       <c r="E49" s="11" t="s">
         <v>458</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="F49" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G49" s="3" t="s">
@@ -5274,20 +5278,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="50" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B50" s="3">
         <v>46</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D50" s="11" t="s">
+      <c r="D50" s="21" t="s">
         <v>509</v>
       </c>
       <c r="E50" s="11" t="s">
         <v>459</v>
       </c>
-      <c r="F50" s="3" t="s">
+      <c r="F50" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G50" s="3" t="s">
@@ -5318,20 +5322,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="51" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B51" s="3">
         <v>47</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D51" s="21" t="s">
         <v>510</v>
       </c>
       <c r="E51" s="11" t="s">
         <v>460</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="F51" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G51" s="3" t="s">
@@ -5362,20 +5366,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="52" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B52" s="3">
         <v>48</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="21" t="s">
         <v>511</v>
       </c>
       <c r="E52" s="11" t="s">
         <v>461</v>
       </c>
-      <c r="F52" s="3" t="s">
+      <c r="F52" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G52" s="3" t="s">
@@ -5406,20 +5410,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="53" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B53" s="3">
         <v>49</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D53" s="11" t="s">
+      <c r="D53" s="21" t="s">
         <v>512</v>
       </c>
       <c r="E53" s="11" t="s">
         <v>462</v>
       </c>
-      <c r="F53" s="3" t="s">
+      <c r="F53" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G53" s="3" t="s">
@@ -5450,20 +5454,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="54" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B54" s="3">
         <v>50</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="21" t="s">
         <v>513</v>
       </c>
       <c r="E54" s="11" t="s">
         <v>463</v>
       </c>
-      <c r="F54" s="3" t="s">
+      <c r="F54" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G54" s="3" t="s">
@@ -5494,20 +5498,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="55" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B55" s="3">
         <v>51</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D55" s="21" t="s">
         <v>523</v>
       </c>
       <c r="E55" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="F55" s="3" t="s">
+      <c r="F55" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G55" s="3" t="s">
@@ -5538,20 +5542,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="56" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B56" s="3">
         <v>52</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="21" t="s">
         <v>524</v>
       </c>
       <c r="E56" s="11" t="s">
         <v>514</v>
       </c>
-      <c r="F56" s="3" t="s">
+      <c r="F56" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G56" s="3" t="s">
@@ -5582,20 +5586,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="57" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B57" s="3">
         <v>53</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D57" s="21" t="s">
         <v>525</v>
       </c>
       <c r="E57" s="11" t="s">
         <v>515</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="F57" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G57" s="3" t="s">
@@ -5626,20 +5630,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="58" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B58" s="3">
         <v>54</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="21" t="s">
         <v>526</v>
       </c>
       <c r="E58" s="11" t="s">
         <v>516</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="F58" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G58" s="3" t="s">
@@ -5670,20 +5674,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="59" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B59" s="3">
         <v>55</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="21" t="s">
         <v>527</v>
       </c>
       <c r="E59" s="11" t="s">
         <v>517</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="F59" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G59" s="3" t="s">
@@ -5714,20 +5718,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="60" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B60" s="3">
         <v>56</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="D60" s="21" t="s">
         <v>528</v>
       </c>
       <c r="E60" s="11" t="s">
         <v>518</v>
       </c>
-      <c r="F60" s="3" t="s">
+      <c r="F60" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G60" s="3" t="s">
@@ -5758,20 +5762,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="61" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B61" s="3">
         <v>57</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D61" s="11" t="s">
+      <c r="D61" s="21" t="s">
         <v>529</v>
       </c>
       <c r="E61" s="11" t="s">
         <v>519</v>
       </c>
-      <c r="F61" s="3" t="s">
+      <c r="F61" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G61" s="3" t="s">
@@ -5802,20 +5806,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="62" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B62" s="3">
         <v>58</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D62" s="11" t="s">
+      <c r="D62" s="21" t="s">
         <v>530</v>
       </c>
       <c r="E62" s="11" t="s">
         <v>520</v>
       </c>
-      <c r="F62" s="3" t="s">
+      <c r="F62" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G62" s="3" t="s">
@@ -5846,20 +5850,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="63" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B63" s="3">
         <v>59</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D63" s="11" t="s">
+      <c r="D63" s="21" t="s">
         <v>531</v>
       </c>
       <c r="E63" s="11" t="s">
         <v>521</v>
       </c>
-      <c r="F63" s="3" t="s">
+      <c r="F63" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G63" s="3" t="s">
@@ -5890,20 +5894,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="64" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B64" s="8">
         <v>60</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D64" s="11" t="s">
+      <c r="D64" s="21" t="s">
         <v>532</v>
       </c>
       <c r="E64" s="11" t="s">
         <v>522</v>
       </c>
-      <c r="F64" s="8" t="s">
+      <c r="F64" s="22" t="s">
         <v>4</v>
       </c>
       <c r="G64" s="8" t="s">
@@ -5934,20 +5938,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="65" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B65" s="3">
         <v>1</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D65" s="11" t="s">
+      <c r="D65" s="21" t="s">
         <v>555</v>
       </c>
       <c r="E65" s="11" t="s">
         <v>533</v>
       </c>
-      <c r="F65" s="3" t="s">
+      <c r="F65" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G65" s="3" t="s">
@@ -5978,20 +5982,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="66" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B66" s="3">
         <v>2</v>
       </c>
       <c r="C66" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D66" s="11" t="s">
+      <c r="D66" s="21" t="s">
         <v>556</v>
       </c>
       <c r="E66" s="11" t="s">
         <v>534</v>
       </c>
-      <c r="F66" s="3" t="s">
+      <c r="F66" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G66" s="3" t="s">
@@ -6022,20 +6026,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="67" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B67" s="3">
         <v>3</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D67" s="11" t="s">
+      <c r="D67" s="21" t="s">
         <v>557</v>
       </c>
       <c r="E67" s="11" t="s">
         <v>535</v>
       </c>
-      <c r="F67" s="3" t="s">
+      <c r="F67" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G67" s="3" t="s">
@@ -6066,20 +6070,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="68" spans="2:24" ht="15.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B68" s="3">
         <v>4</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D68" s="21" t="s">
         <v>558</v>
       </c>
       <c r="E68" s="11" t="s">
         <v>536</v>
       </c>
-      <c r="F68" s="3" t="s">
+      <c r="F68" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G68" s="3" t="s">
@@ -6095,20 +6099,20 @@
         <v>15372000</v>
       </c>
     </row>
-    <row r="69" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B69" s="3">
         <v>5</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D69" s="11" t="s">
+      <c r="D69" s="21" t="s">
         <v>559</v>
       </c>
       <c r="E69" s="11" t="s">
         <v>537</v>
       </c>
-      <c r="F69" s="3" t="s">
+      <c r="F69" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G69" s="3" t="s">
@@ -6120,20 +6124,20 @@
       <c r="T69"/>
       <c r="U69"/>
     </row>
-    <row r="70" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B70" s="3">
         <v>6</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D70" s="11" t="s">
+      <c r="D70" s="21" t="s">
         <v>560</v>
       </c>
       <c r="E70" s="11" t="s">
         <v>538</v>
       </c>
-      <c r="F70" s="3" t="s">
+      <c r="F70" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G70" s="3" t="s">
@@ -6145,20 +6149,20 @@
       <c r="T70"/>
       <c r="U70"/>
     </row>
-    <row r="71" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B71" s="3">
         <v>7</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D71" s="11" t="s">
+      <c r="D71" s="21" t="s">
         <v>561</v>
       </c>
       <c r="E71" s="11" t="s">
         <v>539</v>
       </c>
-      <c r="F71" s="3" t="s">
+      <c r="F71" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G71" s="3" t="s">
@@ -6170,20 +6174,20 @@
       <c r="T71"/>
       <c r="U71"/>
     </row>
-    <row r="72" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B72" s="3">
         <v>8</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D72" s="11" t="s">
+      <c r="D72" s="21" t="s">
         <v>562</v>
       </c>
       <c r="E72" s="11" t="s">
         <v>540</v>
       </c>
-      <c r="F72" s="3" t="s">
+      <c r="F72" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G72" s="3" t="s">
@@ -6195,20 +6199,20 @@
       <c r="T72"/>
       <c r="U72"/>
     </row>
-    <row r="73" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B73" s="3">
         <v>9</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D73" s="11" t="s">
+      <c r="D73" s="21" t="s">
         <v>563</v>
       </c>
       <c r="E73" s="11" t="s">
         <v>541</v>
       </c>
-      <c r="F73" s="3" t="s">
+      <c r="F73" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G73" s="3" t="s">
@@ -6220,20 +6224,20 @@
       <c r="T73"/>
       <c r="U73"/>
     </row>
-    <row r="74" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B74" s="3">
         <v>10</v>
       </c>
       <c r="C74" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D74" s="11" t="s">
+      <c r="D74" s="21" t="s">
         <v>564</v>
       </c>
       <c r="E74" s="11" t="s">
         <v>542</v>
       </c>
-      <c r="F74" s="3" t="s">
+      <c r="F74" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G74" s="3" t="s">
@@ -6245,20 +6249,20 @@
       <c r="T74"/>
       <c r="U74"/>
     </row>
-    <row r="75" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B75" s="3">
         <v>11</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D75" s="11" t="s">
+      <c r="D75" s="21" t="s">
         <v>565</v>
       </c>
       <c r="E75" s="11" t="s">
         <v>543</v>
       </c>
-      <c r="F75" s="3" t="s">
+      <c r="F75" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G75" s="3" t="s">
@@ -6278,13 +6282,13 @@
       <c r="C76" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D76" s="11" t="s">
+      <c r="D76" s="21" t="s">
         <v>566</v>
       </c>
       <c r="E76" s="11" t="s">
         <v>544</v>
       </c>
-      <c r="F76" s="3" t="s">
+      <c r="F76" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G76" s="3" t="s">
@@ -6294,20 +6298,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="77" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B77" s="3">
         <v>13</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D77" s="11" t="s">
+      <c r="D77" s="21" t="s">
         <v>567</v>
       </c>
       <c r="E77" s="11" t="s">
         <v>545</v>
       </c>
-      <c r="F77" s="3" t="s">
+      <c r="F77" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G77" s="3" t="s">
@@ -6317,20 +6321,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="78" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B78" s="3">
         <v>14</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D78" s="11" t="s">
+      <c r="D78" s="21" t="s">
         <v>568</v>
       </c>
       <c r="E78" s="11" t="s">
         <v>546</v>
       </c>
-      <c r="F78" s="3" t="s">
+      <c r="F78" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G78" s="3" t="s">
@@ -6340,20 +6344,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="79" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B79" s="3">
         <v>15</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D79" s="11" t="s">
+      <c r="D79" s="21" t="s">
         <v>569</v>
       </c>
       <c r="E79" s="11" t="s">
         <v>547</v>
       </c>
-      <c r="F79" s="3" t="s">
+      <c r="F79" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G79" s="3" t="s">
@@ -6363,20 +6367,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="80" spans="2:24" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B80" s="3">
         <v>16</v>
       </c>
       <c r="C80" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D80" s="11" t="s">
+      <c r="D80" s="21" t="s">
         <v>570</v>
       </c>
       <c r="E80" s="11" t="s">
         <v>548</v>
       </c>
-      <c r="F80" s="3" t="s">
+      <c r="F80" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G80" s="3" t="s">
@@ -6386,20 +6390,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="81" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B81" s="3">
         <v>17</v>
       </c>
       <c r="C81" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D81" s="11" t="s">
+      <c r="D81" s="21" t="s">
         <v>571</v>
       </c>
       <c r="E81" s="11" t="s">
         <v>549</v>
       </c>
-      <c r="F81" s="3" t="s">
+      <c r="F81" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G81" s="3" t="s">
@@ -6409,20 +6413,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="82" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B82" s="3">
         <v>18</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D82" s="11" t="s">
+      <c r="D82" s="21" t="s">
         <v>572</v>
       </c>
       <c r="E82" s="11" t="s">
         <v>550</v>
       </c>
-      <c r="F82" s="3" t="s">
+      <c r="F82" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G82" s="3" t="s">
@@ -6432,20 +6436,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="83" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B83" s="3">
         <v>19</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D83" s="11" t="s">
+      <c r="D83" s="21" t="s">
         <v>573</v>
       </c>
       <c r="E83" s="11" t="s">
         <v>551</v>
       </c>
-      <c r="F83" s="3" t="s">
+      <c r="F83" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G83" s="3" t="s">
@@ -6462,13 +6466,13 @@
       <c r="C84" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D84" s="11" t="s">
+      <c r="D84" s="21" t="s">
         <v>574</v>
       </c>
       <c r="E84" s="11" t="s">
         <v>552</v>
       </c>
-      <c r="F84" s="3" t="s">
+      <c r="F84" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G84" s="3" t="s">
@@ -6478,20 +6482,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="85" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B85" s="3">
         <v>21</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D85" s="11" t="s">
+      <c r="D85" s="21" t="s">
         <v>575</v>
       </c>
       <c r="E85" s="11" t="s">
         <v>553</v>
       </c>
-      <c r="F85" s="3" t="s">
+      <c r="F85" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G85" s="3" t="s">
@@ -6501,20 +6505,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="86" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B86" s="8">
         <v>22</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D86" s="11" t="s">
+      <c r="D86" s="21" t="s">
         <v>576</v>
       </c>
       <c r="E86" s="11" t="s">
         <v>554</v>
       </c>
-      <c r="F86" s="3" t="s">
+      <c r="F86" s="20" t="s">
         <v>4</v>
       </c>
       <c r="G86" s="3" t="s">
@@ -6524,20 +6528,20 @@
         <v>440000</v>
       </c>
     </row>
-    <row r="87" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B87" s="3">
         <v>1</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D87" s="11" t="s">
+      <c r="D87" s="21" t="s">
         <v>600</v>
       </c>
       <c r="E87" s="11" t="s">
         <v>577</v>
       </c>
-      <c r="F87" s="3">
+      <c r="F87" s="20">
         <v>20</v>
       </c>
       <c r="G87" s="3" t="s">
@@ -6547,20 +6551,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="88" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B88" s="3">
         <v>2</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D88" s="11" t="s">
+      <c r="D88" s="21" t="s">
         <v>601</v>
       </c>
       <c r="E88" s="11" t="s">
         <v>578</v>
       </c>
-      <c r="F88" s="3">
+      <c r="F88" s="20">
         <v>20</v>
       </c>
       <c r="G88" s="3" t="s">
@@ -6570,20 +6574,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="89" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B89" s="3">
         <v>3</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D89" s="11" t="s">
+      <c r="D89" s="21" t="s">
         <v>602</v>
       </c>
       <c r="E89" s="11" t="s">
         <v>579</v>
       </c>
-      <c r="F89" s="3">
+      <c r="F89" s="20">
         <v>20</v>
       </c>
       <c r="G89" s="3" t="s">
@@ -6593,20 +6597,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="90" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B90" s="3">
         <v>4</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D90" s="11" t="s">
+      <c r="D90" s="21" t="s">
         <v>603</v>
       </c>
       <c r="E90" s="11" t="s">
         <v>580</v>
       </c>
-      <c r="F90" s="3">
+      <c r="F90" s="20">
         <v>20</v>
       </c>
       <c r="G90" s="3" t="s">
@@ -6616,20 +6620,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="91" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B91" s="3">
         <v>5</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D91" s="11" t="s">
+      <c r="D91" s="21" t="s">
         <v>604</v>
       </c>
       <c r="E91" s="11" t="s">
         <v>581</v>
       </c>
-      <c r="F91" s="3">
+      <c r="F91" s="20">
         <v>20</v>
       </c>
       <c r="G91" s="3" t="s">
@@ -6639,20 +6643,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="92" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B92" s="3">
         <v>6</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D92" s="11" t="s">
+      <c r="D92" s="21" t="s">
         <v>605</v>
       </c>
       <c r="E92" s="11" t="s">
         <v>582</v>
       </c>
-      <c r="F92" s="3">
+      <c r="F92" s="20">
         <v>20</v>
       </c>
       <c r="G92" s="3" t="s">
@@ -6662,20 +6666,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="93" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B93" s="3">
         <v>7</v>
       </c>
       <c r="C93" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D93" s="11" t="s">
+      <c r="D93" s="21" t="s">
         <v>606</v>
       </c>
       <c r="E93" s="11" t="s">
         <v>583</v>
       </c>
-      <c r="F93" s="3">
+      <c r="F93" s="20">
         <v>20</v>
       </c>
       <c r="G93" s="3" t="s">
@@ -6685,20 +6689,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="94" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B94" s="3">
         <v>8</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D94" s="11" t="s">
+      <c r="D94" s="21" t="s">
         <v>607</v>
       </c>
       <c r="E94" s="11" t="s">
         <v>584</v>
       </c>
-      <c r="F94" s="3">
+      <c r="F94" s="20">
         <v>20</v>
       </c>
       <c r="G94" s="3" t="s">
@@ -6708,20 +6712,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="95" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B95" s="3">
         <v>9</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D95" s="11" t="s">
+      <c r="D95" s="21" t="s">
         <v>608</v>
       </c>
       <c r="E95" s="11" t="s">
         <v>585</v>
       </c>
-      <c r="F95" s="3">
+      <c r="F95" s="20">
         <v>20</v>
       </c>
       <c r="G95" s="3" t="s">
@@ -6731,20 +6735,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="96" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B96" s="3">
         <v>10</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D96" s="11" t="s">
+      <c r="D96" s="21" t="s">
         <v>609</v>
       </c>
       <c r="E96" s="11" t="s">
         <v>586</v>
       </c>
-      <c r="F96" s="3">
+      <c r="F96" s="20">
         <v>20</v>
       </c>
       <c r="G96" s="3" t="s">
@@ -6754,20 +6758,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="97" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B97" s="3">
         <v>11</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D97" s="11" t="s">
+      <c r="D97" s="21" t="s">
         <v>610</v>
       </c>
       <c r="E97" s="11" t="s">
         <v>587</v>
       </c>
-      <c r="F97" s="3">
+      <c r="F97" s="20">
         <v>20</v>
       </c>
       <c r="G97" s="3" t="s">
@@ -6777,20 +6781,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="98" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B98" s="3">
         <v>12</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D98" s="11" t="s">
+      <c r="D98" s="21" t="s">
         <v>611</v>
       </c>
       <c r="E98" s="11" t="s">
         <v>588</v>
       </c>
-      <c r="F98" s="3">
+      <c r="F98" s="20">
         <v>20</v>
       </c>
       <c r="G98" s="3" t="s">
@@ -6800,20 +6804,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="99" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B99" s="3">
         <v>13</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D99" s="11" t="s">
+      <c r="D99" s="21" t="s">
         <v>612</v>
       </c>
       <c r="E99" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="F99" s="3">
+      <c r="F99" s="20">
         <v>20</v>
       </c>
       <c r="G99" s="3" t="s">
@@ -6823,20 +6827,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="100" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B100" s="3">
         <v>14</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D100" s="11" t="s">
+      <c r="D100" s="21" t="s">
         <v>613</v>
       </c>
       <c r="E100" s="11" t="s">
         <v>590</v>
       </c>
-      <c r="F100" s="3">
+      <c r="F100" s="20">
         <v>20</v>
       </c>
       <c r="G100" s="3" t="s">
@@ -6846,20 +6850,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="101" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B101" s="3">
         <v>15</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D101" s="11" t="s">
+      <c r="D101" s="21" t="s">
         <v>614</v>
       </c>
       <c r="E101" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="F101" s="3">
+      <c r="F101" s="20">
         <v>20</v>
       </c>
       <c r="G101" s="3" t="s">
@@ -6869,20 +6873,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="102" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B102" s="3">
         <v>16</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D102" s="11" t="s">
+      <c r="D102" s="21" t="s">
         <v>615</v>
       </c>
       <c r="E102" s="11" t="s">
         <v>592</v>
       </c>
-      <c r="F102" s="3">
+      <c r="F102" s="20">
         <v>20</v>
       </c>
       <c r="G102" s="3" t="s">
@@ -6892,20 +6896,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="103" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B103" s="3">
         <v>17</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D103" s="11" t="s">
+      <c r="D103" s="21" t="s">
         <v>616</v>
       </c>
       <c r="E103" s="11" t="s">
         <v>593</v>
       </c>
-      <c r="F103" s="3">
+      <c r="F103" s="20">
         <v>20</v>
       </c>
       <c r="G103" s="3" t="s">
@@ -6915,20 +6919,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="104" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B104" s="3">
         <v>18</v>
       </c>
       <c r="C104" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D104" s="11" t="s">
+      <c r="D104" s="21" t="s">
         <v>617</v>
       </c>
       <c r="E104" s="11" t="s">
         <v>594</v>
       </c>
-      <c r="F104" s="3">
+      <c r="F104" s="20">
         <v>20</v>
       </c>
       <c r="G104" s="3" t="s">
@@ -6938,20 +6942,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="105" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B105" s="3">
         <v>19</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D105" s="11" t="s">
+      <c r="D105" s="21" t="s">
         <v>618</v>
       </c>
       <c r="E105" s="11" t="s">
         <v>595</v>
       </c>
-      <c r="F105" s="3">
+      <c r="F105" s="20">
         <v>20</v>
       </c>
       <c r="G105" s="3" t="s">
@@ -6961,20 +6965,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="106" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B106" s="3">
         <v>20</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D106" s="11" t="s">
+      <c r="D106" s="21" t="s">
         <v>619</v>
       </c>
       <c r="E106" s="11" t="s">
         <v>596</v>
       </c>
-      <c r="F106" s="3">
+      <c r="F106" s="20">
         <v>20</v>
       </c>
       <c r="G106" s="3" t="s">
@@ -6984,20 +6988,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="107" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B107" s="3">
         <v>21</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D107" s="11" t="s">
+      <c r="D107" s="21" t="s">
         <v>620</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>597</v>
       </c>
-      <c r="F107" s="3">
+      <c r="F107" s="20">
         <v>20</v>
       </c>
       <c r="G107" s="3" t="s">
@@ -7007,20 +7011,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="108" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B108" s="3">
         <v>22</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D108" s="11" t="s">
+      <c r="D108" s="21" t="s">
         <v>621</v>
       </c>
       <c r="E108" s="11" t="s">
         <v>598</v>
       </c>
-      <c r="F108" s="3">
+      <c r="F108" s="20">
         <v>20</v>
       </c>
       <c r="G108" s="3" t="s">
@@ -7030,20 +7034,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="109" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B109" s="3">
         <v>23</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D109" s="11" t="s">
+      <c r="D109" s="21" t="s">
         <v>622</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>599</v>
       </c>
-      <c r="F109" s="3">
+      <c r="F109" s="20">
         <v>20</v>
       </c>
       <c r="G109" s="3" t="s">
@@ -7053,20 +7057,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="110" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B110" s="3">
         <v>24</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D110" s="11" t="s">
+      <c r="D110" s="21" t="s">
         <v>664</v>
       </c>
       <c r="E110" s="11" t="s">
         <v>624</v>
       </c>
-      <c r="F110" s="3">
+      <c r="F110" s="20">
         <v>20</v>
       </c>
       <c r="G110" s="3" t="s">
@@ -7076,20 +7080,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="111" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B111" s="3">
         <v>25</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D111" s="11" t="s">
+      <c r="D111" s="21" t="s">
         <v>665</v>
       </c>
       <c r="E111" s="11" t="s">
         <v>625</v>
       </c>
-      <c r="F111" s="3">
+      <c r="F111" s="20">
         <v>20</v>
       </c>
       <c r="G111" s="3" t="s">
@@ -7099,20 +7103,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="112" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B112" s="3">
         <v>26</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D112" s="11" t="s">
+      <c r="D112" s="21" t="s">
         <v>666</v>
       </c>
       <c r="E112" s="11" t="s">
         <v>626</v>
       </c>
-      <c r="F112" s="3">
+      <c r="F112" s="20">
         <v>20</v>
       </c>
       <c r="G112" s="3" t="s">
@@ -7122,20 +7126,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="113" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B113" s="3">
         <v>27</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D113" s="11" t="s">
+      <c r="D113" s="21" t="s">
         <v>667</v>
       </c>
       <c r="E113" s="11" t="s">
         <v>627</v>
       </c>
-      <c r="F113" s="3">
+      <c r="F113" s="20">
         <v>20</v>
       </c>
       <c r="G113" s="3" t="s">
@@ -7145,20 +7149,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="114" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B114" s="3">
         <v>28</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D114" s="11" t="s">
+      <c r="D114" s="21" t="s">
         <v>668</v>
       </c>
       <c r="E114" s="11" t="s">
         <v>628</v>
       </c>
-      <c r="F114" s="3">
+      <c r="F114" s="20">
         <v>20</v>
       </c>
       <c r="G114" s="3" t="s">
@@ -7168,20 +7172,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="115" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B115" s="3">
         <v>29</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D115" s="11" t="s">
+      <c r="D115" s="21" t="s">
         <v>669</v>
       </c>
       <c r="E115" s="11" t="s">
         <v>629</v>
       </c>
-      <c r="F115" s="3">
+      <c r="F115" s="20">
         <v>20</v>
       </c>
       <c r="G115" s="3" t="s">
@@ -7191,20 +7195,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="116" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B116" s="3">
         <v>30</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D116" s="11" t="s">
+      <c r="D116" s="21" t="s">
         <v>670</v>
       </c>
       <c r="E116" s="11" t="s">
         <v>630</v>
       </c>
-      <c r="F116" s="3">
+      <c r="F116" s="20">
         <v>20</v>
       </c>
       <c r="G116" s="3" t="s">
@@ -7214,20 +7218,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="117" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B117" s="3">
         <v>31</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D117" s="11" t="s">
+      <c r="D117" s="21" t="s">
         <v>671</v>
       </c>
       <c r="E117" s="11" t="s">
         <v>631</v>
       </c>
-      <c r="F117" s="3">
+      <c r="F117" s="20">
         <v>20</v>
       </c>
       <c r="G117" s="3" t="s">
@@ -7237,20 +7241,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="118" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B118" s="3">
         <v>32</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D118" s="11" t="s">
+      <c r="D118" s="21" t="s">
         <v>672</v>
       </c>
       <c r="E118" s="11" t="s">
         <v>632</v>
       </c>
-      <c r="F118" s="3">
+      <c r="F118" s="20">
         <v>20</v>
       </c>
       <c r="G118" s="3" t="s">
@@ -7260,20 +7264,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="119" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B119" s="3">
         <v>33</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D119" s="11" t="s">
+      <c r="D119" s="21" t="s">
         <v>673</v>
       </c>
       <c r="E119" s="11" t="s">
         <v>633</v>
       </c>
-      <c r="F119" s="3">
+      <c r="F119" s="20">
         <v>20</v>
       </c>
       <c r="G119" s="3" t="s">
@@ -7283,20 +7287,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="120" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B120" s="3">
         <v>34</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D120" s="11" t="s">
+      <c r="D120" s="21" t="s">
         <v>674</v>
       </c>
       <c r="E120" s="11" t="s">
         <v>634</v>
       </c>
-      <c r="F120" s="3">
+      <c r="F120" s="20">
         <v>20</v>
       </c>
       <c r="G120" s="3" t="s">
@@ -7313,13 +7317,13 @@
       <c r="C121" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D121" s="11" t="s">
+      <c r="D121" s="21" t="s">
         <v>675</v>
       </c>
       <c r="E121" s="11" t="s">
         <v>635</v>
       </c>
-      <c r="F121" s="3">
+      <c r="F121" s="20">
         <v>20</v>
       </c>
       <c r="G121" s="3" t="s">
@@ -7336,13 +7340,13 @@
       <c r="C122" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D122" s="11" t="s">
+      <c r="D122" s="21" t="s">
         <v>676</v>
       </c>
       <c r="E122" s="11" t="s">
         <v>636</v>
       </c>
-      <c r="F122" s="3">
+      <c r="F122" s="20">
         <v>20</v>
       </c>
       <c r="G122" s="3" t="s">
@@ -7352,20 +7356,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="123" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B123" s="3">
         <v>37</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D123" s="11" t="s">
+      <c r="D123" s="21" t="s">
         <v>677</v>
       </c>
       <c r="E123" s="11" t="s">
         <v>637</v>
       </c>
-      <c r="F123" s="3">
+      <c r="F123" s="20">
         <v>20</v>
       </c>
       <c r="G123" s="3" t="s">
@@ -7375,20 +7379,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="124" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B124" s="3">
         <v>38</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D124" s="11" t="s">
+      <c r="D124" s="21" t="s">
         <v>678</v>
       </c>
       <c r="E124" s="11" t="s">
         <v>638</v>
       </c>
-      <c r="F124" s="3">
+      <c r="F124" s="20">
         <v>20</v>
       </c>
       <c r="G124" s="3" t="s">
@@ -7398,20 +7402,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="125" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B125" s="3">
         <v>39</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D125" s="11" t="s">
+      <c r="D125" s="21" t="s">
         <v>679</v>
       </c>
       <c r="E125" s="11" t="s">
         <v>639</v>
       </c>
-      <c r="F125" s="3">
+      <c r="F125" s="20">
         <v>20</v>
       </c>
       <c r="G125" s="3" t="s">
@@ -7421,20 +7425,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="126" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B126" s="3">
         <v>40</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D126" s="11" t="s">
+      <c r="D126" s="21" t="s">
         <v>680</v>
       </c>
       <c r="E126" s="11" t="s">
         <v>640</v>
       </c>
-      <c r="F126" s="3">
+      <c r="F126" s="20">
         <v>20</v>
       </c>
       <c r="G126" s="3" t="s">
@@ -7444,20 +7448,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="127" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B127" s="3">
         <v>41</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D127" s="11" t="s">
+      <c r="D127" s="21" t="s">
         <v>681</v>
       </c>
       <c r="E127" s="11" t="s">
         <v>641</v>
       </c>
-      <c r="F127" s="3">
+      <c r="F127" s="20">
         <v>20</v>
       </c>
       <c r="G127" s="3" t="s">
@@ -7467,20 +7471,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="128" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B128" s="3">
         <v>42</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D128" s="11" t="s">
+      <c r="D128" s="21" t="s">
         <v>682</v>
       </c>
       <c r="E128" s="11" t="s">
         <v>642</v>
       </c>
-      <c r="F128" s="3">
+      <c r="F128" s="20">
         <v>20</v>
       </c>
       <c r="G128" s="3" t="s">
@@ -7497,13 +7501,13 @@
       <c r="C129" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D129" s="11" t="s">
+      <c r="D129" s="21" t="s">
         <v>683</v>
       </c>
       <c r="E129" s="11" t="s">
         <v>643</v>
       </c>
-      <c r="F129" s="3">
+      <c r="F129" s="20">
         <v>20</v>
       </c>
       <c r="G129" s="3" t="s">
@@ -7520,13 +7524,13 @@
       <c r="C130" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D130" s="11" t="s">
+      <c r="D130" s="21" t="s">
         <v>684</v>
       </c>
       <c r="E130" s="11" t="s">
         <v>644</v>
       </c>
-      <c r="F130" s="3">
+      <c r="F130" s="20">
         <v>20</v>
       </c>
       <c r="G130" s="3" t="s">
@@ -7543,13 +7547,13 @@
       <c r="C131" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D131" s="11" t="s">
+      <c r="D131" s="21" t="s">
         <v>685</v>
       </c>
       <c r="E131" s="11" t="s">
         <v>645</v>
       </c>
-      <c r="F131" s="3">
+      <c r="F131" s="20">
         <v>20</v>
       </c>
       <c r="G131" s="3" t="s">
@@ -7566,13 +7570,13 @@
       <c r="C132" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D132" s="11" t="s">
+      <c r="D132" s="21" t="s">
         <v>686</v>
       </c>
       <c r="E132" s="11" t="s">
         <v>646</v>
       </c>
-      <c r="F132" s="3">
+      <c r="F132" s="20">
         <v>20</v>
       </c>
       <c r="G132" s="3" t="s">
@@ -7582,20 +7586,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="133" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B133" s="3">
         <v>47</v>
       </c>
       <c r="C133" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D133" s="11" t="s">
+      <c r="D133" s="21" t="s">
         <v>687</v>
       </c>
       <c r="E133" s="11" t="s">
         <v>647</v>
       </c>
-      <c r="F133" s="3">
+      <c r="F133" s="20">
         <v>20</v>
       </c>
       <c r="G133" s="3" t="s">
@@ -7605,20 +7609,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="134" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B134" s="3">
         <v>48</v>
       </c>
       <c r="C134" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D134" s="11" t="s">
+      <c r="D134" s="21" t="s">
         <v>688</v>
       </c>
       <c r="E134" s="11" t="s">
         <v>648</v>
       </c>
-      <c r="F134" s="3">
+      <c r="F134" s="20">
         <v>20</v>
       </c>
       <c r="G134" s="3" t="s">
@@ -7628,20 +7632,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="135" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B135" s="3">
         <v>49</v>
       </c>
       <c r="C135" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D135" s="11" t="s">
+      <c r="D135" s="21" t="s">
         <v>689</v>
       </c>
       <c r="E135" s="11" t="s">
         <v>649</v>
       </c>
-      <c r="F135" s="3">
+      <c r="F135" s="20">
         <v>20</v>
       </c>
       <c r="G135" s="3" t="s">
@@ -7651,20 +7655,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="136" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B136" s="3">
         <v>50</v>
       </c>
       <c r="C136" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D136" s="11" t="s">
+      <c r="D136" s="21" t="s">
         <v>690</v>
       </c>
       <c r="E136" s="11" t="s">
         <v>650</v>
       </c>
-      <c r="F136" s="3">
+      <c r="F136" s="20">
         <v>20</v>
       </c>
       <c r="G136" s="3" t="s">
@@ -7674,20 +7678,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="137" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B137" s="3">
         <v>51</v>
       </c>
       <c r="C137" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D137" s="11" t="s">
+      <c r="D137" s="21" t="s">
         <v>691</v>
       </c>
       <c r="E137" s="11" t="s">
         <v>651</v>
       </c>
-      <c r="F137" s="3">
+      <c r="F137" s="20">
         <v>20</v>
       </c>
       <c r="G137" s="3" t="s">
@@ -7697,20 +7701,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="138" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B138" s="3">
         <v>52</v>
       </c>
       <c r="C138" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D138" s="11" t="s">
+      <c r="D138" s="21" t="s">
         <v>692</v>
       </c>
       <c r="E138" s="11" t="s">
         <v>652</v>
       </c>
-      <c r="F138" s="3">
+      <c r="F138" s="20">
         <v>20</v>
       </c>
       <c r="G138" s="3" t="s">
@@ -7720,20 +7724,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="139" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B139" s="3">
         <v>53</v>
       </c>
       <c r="C139" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D139" s="11" t="s">
+      <c r="D139" s="21" t="s">
         <v>693</v>
       </c>
       <c r="E139" s="11" t="s">
         <v>653</v>
       </c>
-      <c r="F139" s="3">
+      <c r="F139" s="20">
         <v>20</v>
       </c>
       <c r="G139" s="3" t="s">
@@ -7743,20 +7747,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="140" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B140" s="3">
         <v>54</v>
       </c>
       <c r="C140" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D140" s="11" t="s">
+      <c r="D140" s="21" t="s">
         <v>694</v>
       </c>
       <c r="E140" s="11" t="s">
         <v>654</v>
       </c>
-      <c r="F140" s="3">
+      <c r="F140" s="20">
         <v>20</v>
       </c>
       <c r="G140" s="3" t="s">
@@ -7773,13 +7777,13 @@
       <c r="C141" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D141" s="11" t="s">
+      <c r="D141" s="21" t="s">
         <v>695</v>
       </c>
       <c r="E141" s="11" t="s">
         <v>655</v>
       </c>
-      <c r="F141" s="3">
+      <c r="F141" s="20">
         <v>20</v>
       </c>
       <c r="G141" s="3" t="s">
@@ -7796,13 +7800,13 @@
       <c r="C142" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D142" s="11" t="s">
+      <c r="D142" s="21" t="s">
         <v>696</v>
       </c>
       <c r="E142" s="11" t="s">
         <v>656</v>
       </c>
-      <c r="F142" s="3">
+      <c r="F142" s="20">
         <v>20</v>
       </c>
       <c r="G142" s="3" t="s">
@@ -7812,20 +7816,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="143" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B143" s="3">
         <v>57</v>
       </c>
       <c r="C143" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D143" s="11" t="s">
+      <c r="D143" s="21" t="s">
         <v>697</v>
       </c>
       <c r="E143" s="11" t="s">
         <v>657</v>
       </c>
-      <c r="F143" s="3">
+      <c r="F143" s="20">
         <v>20</v>
       </c>
       <c r="G143" s="3" t="s">
@@ -7835,20 +7839,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="144" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B144" s="3">
         <v>58</v>
       </c>
       <c r="C144" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D144" s="11" t="s">
+      <c r="D144" s="21" t="s">
         <v>698</v>
       </c>
       <c r="E144" s="11" t="s">
         <v>658</v>
       </c>
-      <c r="F144" s="3">
+      <c r="F144" s="20">
         <v>20</v>
       </c>
       <c r="G144" s="3" t="s">
@@ -7858,20 +7862,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="145" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B145" s="3">
         <v>59</v>
       </c>
       <c r="C145" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D145" s="11" t="s">
+      <c r="D145" s="21" t="s">
         <v>699</v>
       </c>
       <c r="E145" s="11" t="s">
         <v>659</v>
       </c>
-      <c r="F145" s="3">
+      <c r="F145" s="20">
         <v>20</v>
       </c>
       <c r="G145" s="3" t="s">
@@ -7881,20 +7885,20 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="146" spans="2:8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B146" s="3">
         <v>60</v>
       </c>
       <c r="C146" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D146" s="11" t="s">
+      <c r="D146" s="21" t="s">
         <v>700</v>
       </c>
       <c r="E146" s="11" t="s">
         <v>660</v>
       </c>
-      <c r="F146" s="3">
+      <c r="F146" s="20">
         <v>20</v>
       </c>
       <c r="G146" s="3" t="s">
@@ -7911,13 +7915,13 @@
       <c r="C147" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D147" s="11" t="s">
+      <c r="D147" s="21" t="s">
         <v>701</v>
       </c>
       <c r="E147" s="11" t="s">
         <v>661</v>
       </c>
-      <c r="F147" s="3">
+      <c r="F147" s="20">
         <v>20</v>
       </c>
       <c r="G147" s="3" t="s">
@@ -7934,13 +7938,13 @@
       <c r="C148" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D148" s="11" t="s">
+      <c r="D148" s="21" t="s">
         <v>702</v>
       </c>
       <c r="E148" s="11" t="s">
         <v>662</v>
       </c>
-      <c r="F148" s="3">
+      <c r="F148" s="20">
         <v>20</v>
       </c>
       <c r="G148" s="3" t="s">
@@ -7957,13 +7961,13 @@
       <c r="C149" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D149" s="11" t="s">
+      <c r="D149" s="21" t="s">
         <v>703</v>
       </c>
       <c r="E149" s="11" t="s">
         <v>663</v>
       </c>
-      <c r="F149" s="3">
+      <c r="F149" s="20">
         <v>20</v>
       </c>
       <c r="G149" s="3" t="s">
@@ -7973,627 +7977,8 @@
         <v>244000</v>
       </c>
     </row>
-    <row r="153" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D153" s="1" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="154" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D154" s="1" t="s">
-        <v>604</v>
-      </c>
-    </row>
-    <row r="155" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D155" s="1" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="156" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D156" s="1" t="s">
-        <v>618</v>
-      </c>
-    </row>
-    <row r="157" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D157" s="1" t="s">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="158" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D158" s="1" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="159" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D159" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="160" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D160" s="1" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="161" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D161" s="1" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="162" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D162" s="1" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="163" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D163" s="1" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="164" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D164" s="1" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="165" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D165" s="1" t="s">
-        <v>670</v>
-      </c>
-    </row>
-    <row r="166" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D166" s="1" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="167" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D167" s="1" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="168" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D168" s="1" t="s">
-        <v>664</v>
-      </c>
-    </row>
-    <row r="169" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D169" s="1" t="s">
-        <v>622</v>
-      </c>
-    </row>
-    <row r="170" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D170" s="1" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="171" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D171" s="1" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="172" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D172" s="1" t="s">
-        <v>609</v>
-      </c>
-    </row>
-    <row r="173" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D173" s="1" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="174" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D174" s="1" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="175" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D175" s="1" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="176" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D176" s="1" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="177" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D177" s="1" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="178" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D178" s="1" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="179" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D179" s="1" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="180" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D180" s="1" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="181" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D181" s="1" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="182" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D182" s="1" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="183" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D183" s="1" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="184" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D184" s="1" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="185" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D185" s="1" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="186" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D186" s="1" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="187" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D187" s="1" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="188" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D188" s="1" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="189" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D189" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="190" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D190" s="1" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="191" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D191" s="1" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="192" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D192" s="1" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="193" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D193" s="1" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="194" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D194" s="1" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="195" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D195" s="1" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="196" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D196" s="1" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="197" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D197" s="1" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="198" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D198" s="1" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="199" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D199" s="1" t="s">
-        <v>672</v>
-      </c>
-    </row>
-    <row r="200" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D200" s="1" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="201" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D201" s="1" t="s">
-        <v>690</v>
-      </c>
-    </row>
-    <row r="202" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D202" s="1" t="s">
-        <v>689</v>
-      </c>
-    </row>
-    <row r="203" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D203" s="1" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="204" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D204" s="1" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="205" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D205" s="1" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="206" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D206" s="1" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="207" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D207" s="1" t="s">
-        <v>601</v>
-      </c>
-    </row>
-    <row r="208" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D208" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="209" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D209" s="1" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="210" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D210" s="1" t="s">
-        <v>694</v>
-      </c>
-    </row>
-    <row r="211" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D211" s="1" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="212" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D212" s="1" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="213" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D213" s="1" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="214" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D214" s="1" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="215" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D215" s="1" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="216" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D216" s="1" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="217" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D217" s="1" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="218" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D218" s="1" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="219" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D219" s="1" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="220" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D220" s="1" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="221" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D221" s="1" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="222" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D222" s="1" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="223" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D223" s="1" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="224" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D224" s="1" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="225" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D225" s="1" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="226" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D226" s="1" t="s">
-        <v>673</v>
-      </c>
-    </row>
-    <row r="227" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D227" s="1" t="s">
-        <v>674</v>
-      </c>
-    </row>
-    <row r="228" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D228" s="1" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="229" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D229" s="1" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="230" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D230" s="1" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="231" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D231" s="1" t="s">
-        <v>617</v>
-      </c>
-    </row>
-    <row r="232" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D232" s="1" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="233" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D233" s="1" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="234" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D234" s="1" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="235" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D235" s="1" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="236" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D236" s="1" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="237" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D237" s="1" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="238" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D238" s="1" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="239" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D239" s="1" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="240" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D240" s="1" t="s">
-        <v>569</v>
-      </c>
-    </row>
-    <row r="241" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D241" s="1" t="s">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="242" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D242" s="1" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="243" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D243" s="1" t="s">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="244" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D244" s="1" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="245" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D245" s="1" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="246" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D246" s="1" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="247" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D247" s="1" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="248" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D248" s="1" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="249" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D249" s="1" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="250" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D250" s="1" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="251" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D251" s="1" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="252" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D252" s="1" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="253" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D253" s="1" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="254" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D254" s="1" t="s">
-        <v>612</v>
-      </c>
-    </row>
-    <row r="255" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D255" s="1" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="256" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D256" s="1" t="s">
-        <v>620</v>
-      </c>
-    </row>
-    <row r="257" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D257" s="1" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="258" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D258" s="1" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="259" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D259" s="1" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="260" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D260" s="1" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="261" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D261" s="1" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="262" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D262" s="1" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="263" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D263" s="1" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="264" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D264" s="1" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="265" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D265" s="1" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="266" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D266" s="1" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="267" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D267" s="1" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="268" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D268" s="1" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="269" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D269" s="1" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="270" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D270" s="1" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="271" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D271" s="1" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="272" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D272" s="1" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="273" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D273" s="1" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="274" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D274" s="1" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="275" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D275" s="1" t="s">
-        <v>525</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:AA149" xr:uid="{4647F203-D603-477A-835D-7581165CB706}">
-    <filterColumn colId="3">
-      <colorFilter dxfId="2"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A4:AA149" xr:uid="{4647F203-D603-477A-835D-7581165CB706}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D153:D197">
     <sortCondition sortBy="cellColor" ref="D153:D197" dxfId="1"/>
   </sortState>

</xml_diff>